<commit_message>
Analyse: feltforklaring under Excel-hovedtabellen
Tilfoejet en FELTFORKLARING-sektion under tabellen paa "Timer (DK)"-fanen:
detaljeret beskrivelse af hvert eneste felt (alle 14 kolonner), plus en
"Generelt"-blok (enhed, median vs gns, ingen-strategi) og en "Andre faner"-
blok der forklarer felterne paa de oevrige fire faner. Ombrudt tekst,
merged celler, eksplicit raekke-indeks (ws.append-desync rettet, saa intet
felt overskrives).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/analyse_handelstimer_out/handelstimer_mes.xlsx
+++ b/backend/analyse_handelstimer_out/handelstimer_mes.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,11 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="001F3864"/>
     </font>
     <font>
       <color rgb="00006100"/>
@@ -120,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -138,11 +143,18 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,7 +164,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -524,22 +536,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1821,9 +1834,327 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>FELTFORKLARING — hvad hver kolonne betyder</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Time (DK)</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Dansk time-interval i vaegur-tid (Europe/Copenhagen). Fx '15:00-16:00' = al bevaegelse mellem kl. 15:00:00 og 15:59:59 dansk tid, samlet paa tvaers af alle dage. Kilden er ET (US-boers) og konverteres tz-bevidst, saa dansk sommertid (CET&lt;-&gt;CEST) haandteres automatisk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>n (dage)</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Antal dage der bidrager til timen (en observation pr. kalenderdato). Hoej n = mere paalideligt tal. Er n under 30 vurderes timen som 'for lidt data' (graa). Timer med faerre minutter end 30 (vedligeholdelse/weekend-kant) er sorteret fra foerst, saa de ikke traekker gennemsnittet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Median range (pt)</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>PRIMAERT bevaegelsesmaal. Median af (timens high - low) paa tvaers af dagene, i indekspoint. Det typiske spaend timen bevaeger sig i. Retningsloest (siger intet om op/ned). Median frem for gennemsnit, saa enkelte vilde nyhedsdage ikke oppuster tallet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Range ($)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Median range omregnet til dollar: range_pt x $5 (MES = $5 pr. indekspoint). Hvad timens typiske spaend er vaerd i penge pr. kontrakt — den hurtige 'kan det betale sig'-linje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Median |beveg.| (pt)</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Median af |close - open|: hvor langt prisen faktisk endte fra sin start i timen (absolut netto, uden fortegn). Er typisk mindre end range, fordi prisen ofte vender undervejs. Stor forskel range vs. |beveg.| = timen churner (frem og tilbage) snarere end at trende.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Gns. afkast (pt, +/-)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>GENNEMSNIT af (close - open) MED fortegn. Positiv = timen tenderer op over de to aar, negativ = ned. Tal taet paa 0 = ingen retningsbias. Gennemsnit (ikke median) her, fordi vi vil fange systematisk drift, ikke den typiske dag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Median max-op (pt)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Median af (high - open): hvor langt OP timen typisk naaede fra sin aabning. Groft long-potentiale i timen — hvor meget en koeb-position kunne loebe med.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Median max-ned (pt)</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Median af (open - low): hvor langt NED timen typisk naaede fra sin aabning. Groft short-potentiale — hvor meget en salgs-position kunne loebe med.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Churn (pt)</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Median af summen af |1-minuts-afkast| inden i timen = total tilbagelagt vej (close-til-close). Hoej churn + LAV range = meget frem og tilbage om samme niveau (godt for mean-reversion). Hoej range + LAV churn = et enkelt rent spring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Median volumen</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Median antal handlede kontrakter i timen (sum over minutterne, median over dagene). Skiller aegte bevaegelse MED likviditet fra tynde spring: en hoej range paa lav volumen er upaalidelig (svaer at komme ind/ud, bredere spread).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Range p90 (pt)</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>90-percentilen af range paa tvaers af dagene — 'haledagene'. Viser hvor stor timen kan blive paa de ~10% vildeste dage. Stor afstand fra medianen = timen har af og til eksplosive dage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Andel store</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>KONSISTENS-maal i procent: andel af dagene hvor timens range oversteg DAGENS EGEN median-range (paa tvaers af doegnets timer). Hoej = timen er paalideligt en af dagens mest aktive; lav = kun faa dage traekker den op. En stor-men-inkonsistent time nedgraderes et trin i vurderingen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Bias</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Retningstendens ud fra median netto-afkast: LONG hvis klart positiv, SHORT hvis klart negativ, ellers 'neutral'. En lille doedzone (0,5 pt) forhindrer stoej i at blive kaldt en bias. NB: selv en 'bias' er svag paa MES — det er en tendens, ikke en regel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Vurdering</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Trafiklys, samlet dom: GROEN = nok bevaegelse OG konsistent; GUL = moderat, vaelg dine spots; ROED = for stille/upaalidelig; GRAA = for lidt data eller lukket time. Kombinerer en absolut cost-floor (er der overhovedet nok?) med en relativ tercil (bedst vs. resten af doegnet) og nedgraderer inkonsistente timer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Generelt</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Enhed</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Alt i indekspoint (pt). 1 tick = 0.25 pt; 1 pt = $5 pr. MES-kontrakt. $-kolonnen er point x 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Median vs. gennemsnit</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Median er primaer (robust mod enkelte ekstreme dage). Gennemsnit vises hvor det tilfoejer noget (afkast/drift). Stor forskel = faa dage traekker — stol paa medianen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Ingen strategi</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Ren beskrivende historik. INGEN entry/exit, P&amp;L, indikatorer eller forudsigelse. 'Groen' betyder 'her er nok at arbejde med', IKKE 'her tjener man penge'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Andre faner i regnearket</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="45" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Ugedag x time (range)</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Matrix: raekker = de 24 danske timer, kolonner = ugedage. Celletal = median range (pt) for den ugedag+time. Farve = relativ tercil paa tvaers af ugens celler (groen=oeverste tredjedel, gul=midt, roed=nederste, graa=n&lt;30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Ugedag x time (volumen)</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Samme matrix, men celletal = median volumen (kontrakter) og farve = relativ tercil af volumen. Læs sammen med range-matrixen: groen begge steder = bevaegelse MED likviditet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="45" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Split-half</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Robusthedstjek. '1. halvdel'/'2. halvdel' = trafiklys for hver periode (foer/efter midtdatoen). 'Robust?' = samme farve i begge. 'Flag' = 'groen kun i en halvdel' (ikke robust) eller 'skift'. Et moenster der kun findes i det ene aar er ikke til at stole paa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Raa aggregat</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Alle tal ufarvet til egen graving: dk_hour, n, &lt;maal&gt;_med og &lt;maal&gt;_avg for hvert af de 6 maal, vol_med/vol_avg, range_p90, andel_store, bias og level (0=graa, 1=roed, 2=gul, 3=groen).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="46">
+    <mergeCell ref="D35:N35"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="D34:N34"/>
+    <mergeCell ref="A45:N45"/>
+    <mergeCell ref="D46:N46"/>
+    <mergeCell ref="D40:N40"/>
+    <mergeCell ref="D31:N31"/>
     <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="D36:N36"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D52:N52"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="D32:N32"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D41:N41"/>
+    <mergeCell ref="D48:N48"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="D53:N53"/>
+    <mergeCell ref="D47:N47"/>
+    <mergeCell ref="A50:N50"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D43:N43"/>
+    <mergeCell ref="D37:N37"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D30:N30"/>
+    <mergeCell ref="D39:N39"/>
+    <mergeCell ref="D33:N33"/>
+    <mergeCell ref="D42:N42"/>
+    <mergeCell ref="D51:N51"/>
+    <mergeCell ref="D38:N38"/>
+    <mergeCell ref="A28:N28"/>
+    <mergeCell ref="D54:N54"/>
+    <mergeCell ref="A54:C54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1885,12 +2216,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>00:00-01:00</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="11" t="n">
         <v>17.9</v>
       </c>
       <c r="C2" s="4" t="n">
@@ -1908,7 +2239,7 @@
       <c r="G2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>01:00-02:00</t>
         </is>
@@ -1931,7 +2262,7 @@
       <c r="G3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>02:00-03:00</t>
         </is>
@@ -1954,7 +2285,7 @@
       <c r="G4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>03:00-04:00</t>
         </is>
@@ -1977,7 +2308,7 @@
       <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>04:00-05:00</t>
         </is>
@@ -2000,7 +2331,7 @@
       <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>05:00-06:00</t>
         </is>
@@ -2023,7 +2354,7 @@
       <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>06:00-07:00</t>
         </is>
@@ -2046,7 +2377,7 @@
       <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>07:00-08:00</t>
         </is>
@@ -2069,7 +2400,7 @@
       <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>08:00-09:00</t>
         </is>
@@ -2092,7 +2423,7 @@
       <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>09:00-10:00</t>
         </is>
@@ -2115,7 +2446,7 @@
       <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>10:00-11:00</t>
         </is>
@@ -2138,7 +2469,7 @@
       <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>11:00-12:00</t>
         </is>
@@ -2161,7 +2492,7 @@
       <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>12:00-13:00</t>
         </is>
@@ -2184,7 +2515,7 @@
       <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>13:00-14:00</t>
         </is>
@@ -2207,7 +2538,7 @@
       <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>14:00-15:00</t>
         </is>
@@ -2218,134 +2549,134 @@
       <c r="C16" s="4" t="n">
         <v>13.6</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="11" t="n">
         <v>15.2</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="11" t="n">
         <v>18</v>
       </c>
       <c r="G16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>15:00-16:00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="11" t="n">
         <v>25.4</v>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="11" t="n">
         <v>22.8</v>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="11" t="n">
         <v>27.8</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="11" t="n">
         <v>24.2</v>
       </c>
       <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>16:00-17:00</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="11" t="n">
         <v>25.8</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="11" t="n">
         <v>23.2</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="11" t="n">
         <v>29.4</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="11" t="n">
         <v>27.9</v>
       </c>
       <c r="G18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>17:00-18:00</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="11" t="n">
         <v>16.9</v>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="11" t="n">
         <v>18.2</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="11" t="n">
         <v>22.4</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="11" t="n">
         <v>20.4</v>
       </c>
       <c r="G19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>18:00-19:00</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="11" t="n">
         <v>15.4</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="11" t="n">
         <v>17.6</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="11" t="n">
         <v>15.8</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="11" t="n">
         <v>19.8</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="11" t="n">
         <v>17.2</v>
       </c>
       <c r="G20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>19:00-20:00</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="11" t="n">
         <v>14.8</v>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="11" t="n">
         <v>16.2</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="11" t="n">
         <v>16.5</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="11" t="n">
         <v>20.5</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="11" t="n">
         <v>17.5</v>
       </c>
       <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>20:00-21:00</t>
         </is>
@@ -2353,45 +2684,45 @@
       <c r="B22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="11" t="n">
         <v>15.5</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="11" t="n">
         <v>18.5</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="11" t="n">
         <v>20.5</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="11" t="n">
         <v>16.6</v>
       </c>
       <c r="G22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>21:00-22:00</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="11" t="n">
         <v>16.8</v>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="11" t="n">
         <v>16.8</v>
       </c>
       <c r="G23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>22:00-23:00</t>
         </is>
@@ -2414,25 +2745,25 @@
       <c r="G24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>23:00-00:00</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B25" s="12" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="12" t="n">
         <v>11.8</v>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>16.6</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="12" t="n">
         <v>12.1</v>
       </c>
       <c r="F25" s="3" t="n"/>
-      <c r="G25" s="9" t="n">
+      <c r="G25" s="12" t="n">
         <v>31.5</v>
       </c>
     </row>
@@ -2504,7 +2835,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>00:00-01:00</t>
         </is>
@@ -2527,7 +2858,7 @@
       <c r="G2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>01:00-02:00</t>
         </is>
@@ -2550,7 +2881,7 @@
       <c r="G3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>02:00-03:00</t>
         </is>
@@ -2573,7 +2904,7 @@
       <c r="G4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>03:00-04:00</t>
         </is>
@@ -2596,7 +2927,7 @@
       <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>04:00-05:00</t>
         </is>
@@ -2619,7 +2950,7 @@
       <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>05:00-06:00</t>
         </is>
@@ -2642,7 +2973,7 @@
       <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>06:00-07:00</t>
         </is>
@@ -2665,7 +2996,7 @@
       <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>07:00-08:00</t>
         </is>
@@ -2688,7 +3019,7 @@
       <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>08:00-09:00</t>
         </is>
@@ -2711,7 +3042,7 @@
       <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>09:00-10:00</t>
         </is>
@@ -2734,7 +3065,7 @@
       <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>10:00-11:00</t>
         </is>
@@ -2757,7 +3088,7 @@
       <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>11:00-12:00</t>
         </is>
@@ -2780,7 +3111,7 @@
       <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>12:00-13:00</t>
         </is>
@@ -2803,7 +3134,7 @@
       <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>13:00-14:00</t>
         </is>
@@ -2826,7 +3157,7 @@
       <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>14:00-15:00</t>
         </is>
@@ -2837,180 +3168,180 @@
       <c r="C16" s="4" t="n">
         <v>25785</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="11" t="n">
         <v>28704</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="11" t="n">
         <v>30827</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="11" t="n">
         <v>31728</v>
       </c>
       <c r="G16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>15:00-16:00</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="11" t="n">
         <v>131426</v>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="11" t="n">
         <v>129478</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="11" t="n">
         <v>137792</v>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="11" t="n">
         <v>148593</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="11" t="n">
         <v>136434</v>
       </c>
       <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>16:00-17:00</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="11" t="n">
         <v>159597</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="11" t="n">
         <v>172282</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="11" t="n">
         <v>181569</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="11" t="n">
         <v>195354</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="11" t="n">
         <v>185920</v>
       </c>
       <c r="G18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>17:00-18:00</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="11" t="n">
         <v>102256</v>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="11" t="n">
         <v>118670</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="11" t="n">
         <v>121884</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="11" t="n">
         <v>141238</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="11" t="n">
         <v>127752</v>
       </c>
       <c r="G19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>18:00-19:00</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="11" t="n">
         <v>77322</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="11" t="n">
         <v>91060</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="11" t="n">
         <v>89153</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="11" t="n">
         <v>98624</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="11" t="n">
         <v>99544</v>
       </c>
       <c r="G20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>19:00-20:00</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="11" t="n">
         <v>73230</v>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="11" t="n">
         <v>82016</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="11" t="n">
         <v>81963</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="11" t="n">
         <v>94684</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="11" t="n">
         <v>85504</v>
       </c>
       <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>20:00-21:00</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="11" t="n">
         <v>71706</v>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="11" t="n">
         <v>75825</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="11" t="n">
         <v>85360</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="11" t="n">
         <v>96454</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="11" t="n">
         <v>84516</v>
       </c>
       <c r="G22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>21:00-22:00</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="11" t="n">
         <v>96924</v>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="11" t="n">
         <v>101258</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="11" t="n">
         <v>107126</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="11" t="n">
         <v>104224</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="11" t="n">
         <v>108844</v>
       </c>
       <c r="G23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>22:00-23:00</t>
         </is>
@@ -3033,25 +3364,25 @@
       <c r="G24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>23:00-00:00</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B25" s="12" t="n">
         <v>6372</v>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="12" t="n">
         <v>7974</v>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>18101</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="12" t="n">
         <v>13433</v>
       </c>
       <c r="F25" s="3" t="n"/>
-      <c r="G25" s="9" t="n">
+      <c r="G25" s="12" t="n">
         <v>37114</v>
       </c>
     </row>
@@ -3123,12 +3454,12 @@
           <t>00:00-01:00</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
@@ -3146,12 +3477,12 @@
           <t>01:00-02:00</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3169,12 +3500,12 @@
           <t>02:00-03:00</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3192,12 +3523,12 @@
           <t>03:00-04:00</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3215,12 +3546,12 @@
           <t>04:00-05:00</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3238,12 +3569,12 @@
           <t>05:00-06:00</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3261,12 +3592,12 @@
           <t>06:00-07:00</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3284,12 +3615,12 @@
           <t>07:00-08:00</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3307,12 +3638,12 @@
           <t>08:00-09:00</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3330,12 +3661,12 @@
           <t>09:00-10:00</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
@@ -3353,17 +3684,17 @@
           <t>10:00-11:00</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>NEJ</t>
         </is>
@@ -3380,12 +3711,12 @@
           <t>11:00-12:00</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3403,12 +3734,12 @@
           <t>12:00-13:00</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3426,12 +3757,12 @@
           <t>13:00-14:00</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>🟡</t>
         </is>
@@ -3449,12 +3780,12 @@
           <t>14:00-15:00</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3472,12 +3803,12 @@
           <t>15:00-16:00</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3495,12 +3826,12 @@
           <t>16:00-17:00</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3518,12 +3849,12 @@
           <t>17:00-18:00</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3541,12 +3872,12 @@
           <t>18:00-19:00</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3564,12 +3895,12 @@
           <t>19:00-20:00</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3587,12 +3918,12 @@
           <t>20:00-21:00</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3610,12 +3941,12 @@
           <t>21:00-22:00</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>🟢</t>
         </is>
@@ -3633,12 +3964,12 @@
           <t>22:00-23:00</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>🔴</t>
         </is>
@@ -3656,12 +3987,12 @@
           <t>23:00-00:00</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>⚪</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>⚪</t>
         </is>

</xml_diff>